<commit_message>
Add AWS Rekognition Face Liveness
</commit_message>
<xml_diff>
--- a/public/TemplateExcel/Class.xlsx
+++ b/public/TemplateExcel/Class.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\buiho\OneDrive\Máy tính\TemplateExcel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DoAn\EduAttend\fe\public\TemplateExcel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{497D557C-A355-43AA-BE54-7E21D6EA9B38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2980F0E7-2C63-4CFA-A0DE-B869DEA45FD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -90,7 +90,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -98,12 +98,28 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -393,101 +409,101 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="1" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="1" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="1" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+      <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="1" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+      <c r="A6" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="1" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+      <c r="A7" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="1" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+      <c r="A8" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="1" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+      <c r="A9" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="1" t="s">
         <v>0</v>
       </c>
     </row>

</xml_diff>